<commit_message>
Update: Threat Alert Report - 2026-03-30 02:40
</commit_message>
<xml_diff>
--- a/excel_routes/route_ATZ_JED_threats.xlsx
+++ b/excel_routes/route_ATZ_JED_threats.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -523,27 +523,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>25-MAR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SM-453</t>
+          <t>SM-455</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-452</t>
+          <t>Nesma Airlines NE-170</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>3983</v>
+        <v>4040</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4094</v>
+        <v>7884</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-111</v>
+        <v>-3844</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -568,27 +568,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>25-MAR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SM-453</t>
+          <t>SM-455</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-450</t>
+          <t>Nile Air NP-529</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3983</v>
+        <v>4082</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4094</v>
+        <v>7884</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-111</v>
+        <v>-3802</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -613,27 +613,27 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>27-MAR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SM-491</t>
+          <t>SM-455</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-452</t>
+          <t>Nile Air NP-629</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>6740</v>
+        <v>4082</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>7512</v>
+        <v>7884</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-772</v>
+        <v>-3802</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>30</v>
@@ -658,27 +658,27 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>27-MAR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SM-953</t>
+          <t>SM-455</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-452</t>
+          <t>Nile Air NP-627</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>6740</v>
+        <v>4082</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>7044</v>
+        <v>7884</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-304</v>
+        <v>-3802</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>30</v>
@@ -703,7 +703,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>01-APR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -713,17 +713,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-530</t>
+          <t>Nile Air NP-427</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5059</v>
+        <v>4082</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>6575</v>
+        <v>7884</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-1516</v>
+        <v>-3802</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>30</v>
@@ -748,7 +748,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>01-APR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -758,17 +758,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-578</t>
+          <t>Nile Air NP-127</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5059</v>
+        <v>4082</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6575</v>
+        <v>7884</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-1516</v>
+        <v>-3802</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>30</v>
@@ -793,7 +793,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>01-APR-26</t>
+          <t>30-MAR-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -803,17 +803,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-576</t>
+          <t>Nile Air NP-227</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>5059</v>
+        <v>4082</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>6575</v>
+        <v>7884</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-1516</v>
+        <v>-3802</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>30</v>
@@ -838,7 +838,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>03-APR-26</t>
+          <t>31-MAR-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -848,17 +848,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-578</t>
+          <t>Nesma Airlines NE-178</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>3983</v>
+        <v>4040</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>6575</v>
+        <v>6930</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-2592</v>
+        <v>-2890</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>30</v>
@@ -883,7 +883,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>03-APR-26</t>
+          <t>31-MAR-26</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -893,17 +893,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-576</t>
+          <t>Nesma Airlines NE-970</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>3983</v>
+        <v>4040</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>6575</v>
+        <v>6930</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-2592</v>
+        <v>-2890</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>30</v>
@@ -928,7 +928,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>04-APR-26</t>
+          <t>31-MAR-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -938,26 +938,26 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-673</t>
+          <t>Nile Air NP-227</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6286</v>
+        <v>4082</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>7044</v>
+        <v>6930</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-758</v>
+        <v>-2848</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>04-APR-26</t>
+          <t>31-MAR-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -983,26 +983,26 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-665</t>
+          <t>Nile Air NP-329</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>6286</v>
+        <v>4082</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>7044</v>
+        <v>6930</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-758</v>
+        <v>-2848</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>04-APR-26</t>
+          <t>31-MAR-26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1028,33 +1028,663 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>EgyptAir MS-643</t>
+          <t>Nile Air NP-527</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6396</v>
+        <v>4082</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>7044</v>
+        <v>6930</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-648</v>
+        <v>-2848</v>
       </c>
       <c r="G13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>31-MAR-26</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-327</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>4082</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>6930</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>-2848</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>31-MAR-26</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-127</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>4082</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>6930</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>-2848</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>01-APR-26</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-530</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>5120</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>6158</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>-1038</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>01-APR-26</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-578</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>5120</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>6158</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>-1038</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>01-APR-26</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-576</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>5120</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>6158</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>-1038</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>03-APR-26</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-578</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>6242</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>7407</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>-1165</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>03-APR-26</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-576</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>6242</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>7407</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>-1165</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>05-APR-26</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-174</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>4040</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>6930</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>-2890</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>06-APR-26</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-669</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>6369</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>7407</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>-1038</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I13" s="2" t="n">
+      <c r="H22" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I22" s="2" t="n">
         <v>-16</v>
       </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>LOW THREAT</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>07-APR-26</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-669</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>6369</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>6930</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>-561</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>11-MAY-26</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>flynas XY-574</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>6860</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>9680</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>-2820</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>11-MAY-26</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>flynas XY-584</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>6860</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>9680</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>-2820</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>11-MAY-26</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>flynas XY-570</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>6860</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>9680</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>-2820</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>11-MAY-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>flynas XY-572</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>6860</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>9680</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>-2820</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>LOW THREAT</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>EGP</t>
         </is>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-17 20:44
</commit_message>
<xml_diff>
--- a/excel_routes/route_ATZ_JED_threats.xlsx
+++ b/excel_routes/route_ATZ_JED_threats.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -610,6 +610,51 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>21-MAY-26</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-170</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>5058</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>8919</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>-3861</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update: Threat Alert Report - 2026-05-22 11:34
</commit_message>
<xml_diff>
--- a/excel_routes/route_ATZ_JED_threats.xlsx
+++ b/excel_routes/route_ATZ_JED_threats.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>29-MAY-26</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-170</t>
+          <t>Nesma Airlines NE-174</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>3722</v>
+        <v>6214</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7488</v>
+        <v>11076</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-3766</v>
+        <v>-4862</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>30</v>
@@ -586,7 +586,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>29-MAY-26</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -596,17 +596,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-174</t>
+          <t>Nile Air NP-127</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>3722</v>
+        <v>7821</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>7488</v>
+        <v>11076</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-3766</v>
+        <v>-3255</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>30</v>
@@ -631,7 +631,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>25-MAY-26</t>
+          <t>29-MAY-26</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -641,26 +641,26 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-327</t>
+          <t>flynas XY-568</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3892</v>
+        <v>8638</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>7488</v>
+        <v>11076</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>-3596</v>
+        <v>-2438</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>29-MAY-26</t>
+          <t>03-JUN-26</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -686,17 +686,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-174</t>
+          <t>Nesma Airlines NE-170</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>6228</v>
+        <v>6214</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>11084</v>
+        <v>16699</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-4856</v>
+        <v>-10485</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>30</v>
@@ -707,9 +707,9 @@
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>29-MAY-26</t>
+          <t>03-JUN-26</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-127</t>
+          <t>Nesma Airlines NE-172</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7856</v>
+        <v>6214</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>11084</v>
+        <v>16699</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-3228</v>
+        <v>-10485</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>30</v>
@@ -752,9 +752,9 @@
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -776,17 +776,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-170</t>
+          <t>Nile Air NP-227</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>6228</v>
+        <v>6355</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>16718</v>
+        <v>16699</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>-10490</v>
+        <v>-10344</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>30</v>
@@ -811,7 +811,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>03-JUN-26</t>
+          <t>04-JUN-26</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -821,30 +821,30 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-172</t>
+          <t>EgyptAir MS-673</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>6228</v>
+        <v>5792</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>16718</v>
+        <v>13402</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-10490</v>
+        <v>-7610</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>30</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>7</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>03-JUN-26</t>
+          <t>04-JUN-26</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -870,13 +870,13 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>6384</v>
+        <v>6355</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>16718</v>
+        <v>13402</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-10334</v>
+        <v>-7047</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>30</v>
@@ -887,9 +887,9 @@
       <c r="I9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -911,17 +911,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-170</t>
+          <t>Nile Air NP-127</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>6228</v>
+        <v>6355</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>13419</v>
+        <v>13402</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>-7191</v>
+        <v>-7047</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>30</v>
@@ -946,7 +946,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>04-JUN-26</t>
+          <t>07-JUN-26</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -956,17 +956,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Nesma Airlines NE-172</t>
+          <t>Nesma Airlines NE-170</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6228</v>
+        <v>6214</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>13419</v>
+        <v>13402</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-7191</v>
+        <v>-7188</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>30</v>
@@ -991,7 +991,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>04-JUN-26</t>
+          <t>07-JUN-26</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1001,17 +1001,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Nile Air NP-227</t>
+          <t>Nesma Airlines NE-172</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>6384</v>
+        <v>6214</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>13419</v>
+        <v>13402</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-7035</v>
+        <v>-7188</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>30</v>
@@ -1028,6 +1028,591 @@
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>07-JUN-26</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-127</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>6355</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>13402</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>-7047</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>08-JUN-26</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-643</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>08-JUN-26</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-641</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>08-JUN-26</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-655</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>09-JUN-26</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-170</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>6214</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>-5933</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>09-JUN-26</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Nile Air NP-227</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>6355</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>-5792</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>09-JUN-26</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-655</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>10-JUN-26</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-643</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>10-JUN-26</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-641</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>10-JUN-26</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-665</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>12147</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>-3889</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>11-JUN-26</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Nesma Airlines NE-176</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>6214</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>9568</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>-3354</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>11-JUN-26</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-643</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>9568</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>-1310</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>EGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>11-JUN-26</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>SM-455</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>EgyptAir MS-641</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>8258</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>9568</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>-1310</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>-16</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>EGP</t>
         </is>

</xml_diff>